<commit_message>
Respaldo local antes de forzar subida
</commit_message>
<xml_diff>
--- a/Jira/Plan de Prueba para Jira_y_Reportes de Bug/Modulo_Gestión de Transferencia/Plantilla de Test Cases_Gestión de Transferencia -v 3.0.xlsx
+++ b/Jira/Plan de Prueba para Jira_y_Reportes de Bug/Modulo_Gestión de Transferencia/Plantilla de Test Cases_Gestión de Transferencia -v 3.0.xlsx
@@ -5,11 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Desktop\Portafolio\Plan de Prueba para Jira_y_Reportes de Bug\Modulo_Gestión de Transferencia\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Desktop\Portafolio\Jira\Plan de Prueba para Jira_y_Reportes de Bug\Modulo_Gestión de Transferencia\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="fSgyRIZMtfWVL4fHA4hogEdtf/RbFExjiMmNhcAd/KAubYVoeWKqUoxc4jl2eMez81vJ05SkrBqJ+cunfTZE9Q==" workbookSaltValue="M1scwkW0RGi/G72+5SeYHQ==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11715" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11715" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Información" sheetId="7" r:id="rId1"/>
@@ -2883,6 +2884,7 @@
       <c r="K21" s="74"/>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="GshwpZ1u3jCwPH4GDjx4wczJ/Z/G+FvdnbsF0fwwXkRRAkG0/p+9qMRfPu9wXvqFpjMDAiK+cbgCGdUy6WLE1Q==" saltValue="PPxVZQsu5vD+514+QazE/Q==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <mergeCells count="4">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
@@ -3204,6 +3206,7 @@
       <c r="W4" s="50"/>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="0t/s17lPbe4+fWlgq02IljNYXxv2a0a2cqy4mIaGiIB5WlEAlAa6KfQt9FK5dCJAB6crKGZoaBQqhKLWnfTPCA==" saltValue="xW6UWC0+55NW7mICA+6Kmw==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <conditionalFormatting sqref="O2">
     <cfRule type="cellIs" dxfId="14" priority="11" operator="equal">
       <formula>"Crítico"</formula>
@@ -4365,6 +4368,7 @@
       <c r="G121" s="99"/>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="eL9sw/aSPfocmfa5jx8e2xa9v0XIBIliIwFWTooRXK1YTH3QJYozL/OBY7cao5bu6dDA+85tJ3ic0293xTQX5w==" saltValue="clEHaHehhbGKCh5Lrevn2Q==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <mergeCells count="7">
     <mergeCell ref="A2:G6"/>
     <mergeCell ref="A85:G85"/>
@@ -5195,6 +5199,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="mv1pM/0r6OmolenHID3ibUIOOcgfqHYDf03nb0u063hVyxidZK5fNmzFHgmecISe0XbqZMPjIVKc6MzgE6q0sA==" saltValue="WsWkIuJ4T5wWb+SDxozp/Q==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <mergeCells count="5">
     <mergeCell ref="A77:A78"/>
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
Reparando estructura de carpetas y añadiendo archivos
</commit_message>
<xml_diff>
--- a/Jira/Plan de Prueba para Jira_y_Reportes de Bug/Modulo_Gestión de Transferencia/Plantilla de Test Cases_Gestión de Transferencia -v 3.0.xlsx
+++ b/Jira/Plan de Prueba para Jira_y_Reportes de Bug/Modulo_Gestión de Transferencia/Plantilla de Test Cases_Gestión de Transferencia -v 3.0.xlsx
@@ -8,7 +8,6 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Desktop\Portafolio\Jira\Plan de Prueba para Jira_y_Reportes de Bug\Modulo_Gestión de Transferencia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="fSgyRIZMtfWVL4fHA4hogEdtf/RbFExjiMmNhcAd/KAubYVoeWKqUoxc4jl2eMez81vJ05SkrBqJ+cunfTZE9Q==" workbookSaltValue="M1scwkW0RGi/G72+5SeYHQ==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11715" activeTab="3"/>
   </bookViews>
@@ -1057,7 +1056,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="37">
+  <fonts count="37" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1759,7 +1758,7 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="105">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2061,6 +2060,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2773,9 +2784,9 @@
     <tabColor theme="8"/>
   </sheetPr>
   <dimension ref="A1:K21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:10" ht="22.5">
+    <row r="1" spans="1:10" ht="22.5" x14ac:dyDescent="0.2">
       <c r="A1" s="77" t="s">
         <v>208</v>
       </c>
@@ -2785,7 +2796,7 @@
       <c r="E1" s="77"/>
       <c r="F1" s="77"/>
     </row>
-    <row r="2" spans="1:10" ht="18">
+    <row r="2" spans="1:10" ht="18" x14ac:dyDescent="0.2">
       <c r="A2" s="78" t="s">
         <v>209</v>
       </c>
@@ -2795,30 +2806,30 @@
       <c r="E2" s="78"/>
       <c r="F2" s="78"/>
     </row>
-    <row r="4" spans="1:10" ht="14.25">
+    <row r="4" spans="1:10" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A4" s="71" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="14.25">
+    <row r="5" spans="1:10" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A5" s="71" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="29.25">
+    <row r="8" spans="1:10" ht="29.25" x14ac:dyDescent="0.2">
       <c r="A8" s="72" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="9" spans="1:10" s="1" customFormat="1" ht="29.25">
+    <row r="9" spans="1:10" s="1" customFormat="1" ht="29.25" x14ac:dyDescent="0.2">
       <c r="A9" s="72"/>
     </row>
-    <row r="10" spans="1:10" ht="22.5" thickBot="1">
+    <row r="10" spans="1:10" ht="22.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="73" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="59.25" customHeight="1" thickBot="1">
+    <row r="11" spans="1:10" ht="59.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="79" t="s">
         <v>216</v>
       </c>
@@ -2830,15 +2841,15 @@
       <c r="G11" s="81"/>
       <c r="J11" s="74"/>
     </row>
-    <row r="12" spans="1:10" s="1" customFormat="1" ht="14.25">
+    <row r="12" spans="1:10" s="1" customFormat="1" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A12" s="63"/>
     </row>
-    <row r="13" spans="1:10" ht="22.5" thickBot="1">
+    <row r="13" spans="1:10" ht="22.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="73" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="48.75" customHeight="1" thickBot="1">
+    <row r="14" spans="1:10" ht="48.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="79" t="s">
         <v>223</v>
       </c>
@@ -2849,20 +2860,20 @@
       <c r="F14" s="80"/>
       <c r="G14" s="81"/>
     </row>
-    <row r="15" spans="1:10" s="1" customFormat="1" ht="14.25">
+    <row r="15" spans="1:10" s="1" customFormat="1" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A15" s="63"/>
     </row>
-    <row r="16" spans="1:10" ht="21.75">
+    <row r="16" spans="1:10" ht="21.75" x14ac:dyDescent="0.2">
       <c r="A16" s="73" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="14.25">
+    <row r="17" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A17" s="71" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="18" spans="1:11" s="1" customFormat="1" ht="14.25">
+    <row r="18" spans="1:11" s="1" customFormat="1" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A18" s="75" t="s">
         <v>217</v>
       </c>
@@ -2870,21 +2881,21 @@
       <c r="C18" s="76"/>
       <c r="D18" s="76"/>
     </row>
-    <row r="19" spans="1:11" ht="14.25">
+    <row r="19" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A19" s="71" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="14.25">
+    <row r="20" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A20" s="70" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="21" spans="1:11">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="K21" s="74"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="GshwpZ1u3jCwPH4GDjx4wczJ/Z/G+FvdnbsF0fwwXkRRAkG0/p+9qMRfPu9wXvqFpjMDAiK+cbgCGdUy6WLE1Q==" saltValue="PPxVZQsu5vD+514+QazE/Q==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <mergeCells count="4">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
@@ -2904,7 +2915,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:X4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" style="62" customWidth="1"/>
     <col min="2" max="2" width="17.7109375" style="52" customWidth="1"/>
@@ -2924,7 +2935,7 @@
     <col min="25" max="16384" width="12.5703125" style="52"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="36">
+    <row r="1" spans="1:24" ht="36" x14ac:dyDescent="0.2">
       <c r="A1" s="61" t="s">
         <v>21</v>
       </c>
@@ -2998,7 +3009,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="2" spans="1:24" ht="227.25" customHeight="1">
+    <row r="2" spans="1:24" ht="227.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>46087</v>
       </c>
@@ -3067,7 +3078,7 @@
       </c>
       <c r="W2" s="50"/>
     </row>
-    <row r="3" spans="1:24" ht="279.75" customHeight="1">
+    <row r="3" spans="1:24" ht="279.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>46087</v>
       </c>
@@ -3138,7 +3149,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="4" spans="1:24" ht="409.5">
+    <row r="4" spans="1:24" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>46088</v>
       </c>
@@ -3206,7 +3217,7 @@
       <c r="W4" s="50"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="0t/s17lPbe4+fWlgq02IljNYXxv2a0a2cqy4mIaGiIB5WlEAlAa6KfQt9FK5dCJAB6crKGZoaBQqhKLWnfTPCA==" saltValue="xW6UWC0+55NW7mICA+6Kmw==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <conditionalFormatting sqref="O2">
     <cfRule type="cellIs" dxfId="14" priority="11" operator="equal">
       <formula>"Crítico"</formula>
@@ -3297,7 +3308,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup paperSize="9" fitToHeight="0" pageOrder="overThenDown" orientation="landscape" cellComments="atEnd" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="17" fitToHeight="0" pageOrder="overThenDown" orientation="landscape" cellComments="atEnd" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3307,12 +3318,12 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A2:H121"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="7" max="7" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" hidden="1">
+    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" s="82"/>
       <c r="B2" s="83"/>
       <c r="C2" s="83"/>
@@ -3321,7 +3332,7 @@
       <c r="F2" s="83"/>
       <c r="G2" s="84"/>
     </row>
-    <row r="3" spans="1:7" hidden="1">
+    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" s="82"/>
       <c r="B3" s="83"/>
       <c r="C3" s="83"/>
@@ -3330,7 +3341,7 @@
       <c r="F3" s="83"/>
       <c r="G3" s="84"/>
     </row>
-    <row r="4" spans="1:7" hidden="1">
+    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" s="82"/>
       <c r="B4" s="83"/>
       <c r="C4" s="83"/>
@@ -3339,7 +3350,7 @@
       <c r="F4" s="83"/>
       <c r="G4" s="84"/>
     </row>
-    <row r="5" spans="1:7" hidden="1">
+    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" s="82"/>
       <c r="B5" s="83"/>
       <c r="C5" s="83"/>
@@ -3348,7 +3359,7 @@
       <c r="F5" s="83"/>
       <c r="G5" s="84"/>
     </row>
-    <row r="6" spans="1:7" ht="13.5" hidden="1" thickBot="1">
+    <row r="6" spans="1:7" ht="13.5" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="85"/>
       <c r="B6" s="86"/>
       <c r="C6" s="86"/>
@@ -3357,9 +3368,9 @@
       <c r="F6" s="86"/>
       <c r="G6" s="87"/>
     </row>
-    <row r="7" spans="1:7" hidden="1"/>
-    <row r="8" spans="1:7" ht="13.5" thickBot="1"/>
-    <row r="9" spans="1:7" ht="21" thickBot="1">
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.2"/>
+    <row r="8" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="1:7" ht="21" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="88" t="s">
         <v>25</v>
       </c>
@@ -3370,7 +3381,7 @@
       <c r="F9" s="89"/>
       <c r="G9" s="90"/>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="91"/>
       <c r="B10" s="92"/>
       <c r="C10" s="92"/>
@@ -3379,7 +3390,7 @@
       <c r="F10" s="92"/>
       <c r="G10" s="93"/>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="94"/>
       <c r="B11" s="95"/>
       <c r="C11" s="95"/>
@@ -3388,7 +3399,7 @@
       <c r="F11" s="95"/>
       <c r="G11" s="96"/>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="94"/>
       <c r="B12" s="95"/>
       <c r="C12" s="95"/>
@@ -3397,7 +3408,7 @@
       <c r="F12" s="95"/>
       <c r="G12" s="96"/>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="94"/>
       <c r="B13" s="95"/>
       <c r="C13" s="95"/>
@@ -3406,7 +3417,7 @@
       <c r="F13" s="95"/>
       <c r="G13" s="96"/>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="94"/>
       <c r="B14" s="95"/>
       <c r="C14" s="95"/>
@@ -3415,7 +3426,7 @@
       <c r="F14" s="95"/>
       <c r="G14" s="96"/>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="94"/>
       <c r="B15" s="95"/>
       <c r="C15" s="95"/>
@@ -3424,7 +3435,7 @@
       <c r="F15" s="95"/>
       <c r="G15" s="96"/>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="94"/>
       <c r="B16" s="95"/>
       <c r="C16" s="95"/>
@@ -3433,7 +3444,7 @@
       <c r="F16" s="95"/>
       <c r="G16" s="96"/>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="94"/>
       <c r="B17" s="95"/>
       <c r="C17" s="95"/>
@@ -3442,7 +3453,7 @@
       <c r="F17" s="95"/>
       <c r="G17" s="96"/>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="94"/>
       <c r="B18" s="95"/>
       <c r="C18" s="95"/>
@@ -3451,7 +3462,7 @@
       <c r="F18" s="95"/>
       <c r="G18" s="96"/>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="94"/>
       <c r="B19" s="95"/>
       <c r="C19" s="95"/>
@@ -3460,7 +3471,7 @@
       <c r="F19" s="95"/>
       <c r="G19" s="96"/>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="94"/>
       <c r="B20" s="95"/>
       <c r="C20" s="95"/>
@@ -3469,7 +3480,7 @@
       <c r="F20" s="95"/>
       <c r="G20" s="96"/>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" s="94"/>
       <c r="B21" s="95"/>
       <c r="C21" s="95"/>
@@ -3478,7 +3489,7 @@
       <c r="F21" s="95"/>
       <c r="G21" s="96"/>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" s="94"/>
       <c r="B22" s="95"/>
       <c r="C22" s="95"/>
@@ -3487,7 +3498,7 @@
       <c r="F22" s="95"/>
       <c r="G22" s="96"/>
     </row>
-    <row r="23" spans="1:7">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" s="94"/>
       <c r="B23" s="95"/>
       <c r="C23" s="95"/>
@@ -3496,7 +3507,7 @@
       <c r="F23" s="95"/>
       <c r="G23" s="96"/>
     </row>
-    <row r="24" spans="1:7">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="94"/>
       <c r="B24" s="95"/>
       <c r="C24" s="95"/>
@@ -3505,7 +3516,7 @@
       <c r="F24" s="95"/>
       <c r="G24" s="96"/>
     </row>
-    <row r="25" spans="1:7">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -3514,7 +3525,7 @@
       <c r="F25" s="95"/>
       <c r="G25" s="96"/>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" s="94"/>
       <c r="B26" s="95"/>
       <c r="C26" s="95"/>
@@ -3523,7 +3534,7 @@
       <c r="F26" s="95"/>
       <c r="G26" s="96"/>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" s="94"/>
       <c r="B27" s="95"/>
       <c r="C27" s="95"/>
@@ -3532,7 +3543,7 @@
       <c r="F27" s="95"/>
       <c r="G27" s="96"/>
     </row>
-    <row r="28" spans="1:7">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" s="94"/>
       <c r="B28" s="95"/>
       <c r="C28" s="95"/>
@@ -3541,7 +3552,7 @@
       <c r="F28" s="95"/>
       <c r="G28" s="96"/>
     </row>
-    <row r="29" spans="1:7">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" s="94"/>
       <c r="B29" s="95"/>
       <c r="C29" s="95"/>
@@ -3550,7 +3561,7 @@
       <c r="F29" s="95"/>
       <c r="G29" s="96"/>
     </row>
-    <row r="30" spans="1:7">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" s="94"/>
       <c r="B30" s="95"/>
       <c r="C30" s="95"/>
@@ -3559,7 +3570,7 @@
       <c r="F30" s="95"/>
       <c r="G30" s="96"/>
     </row>
-    <row r="31" spans="1:7">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" s="94"/>
       <c r="B31" s="95"/>
       <c r="C31" s="95"/>
@@ -3568,7 +3579,7 @@
       <c r="F31" s="95"/>
       <c r="G31" s="96"/>
     </row>
-    <row r="32" spans="1:7">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" s="94"/>
       <c r="B32" s="95"/>
       <c r="C32" s="95"/>
@@ -3577,7 +3588,7 @@
       <c r="F32" s="95"/>
       <c r="G32" s="96"/>
     </row>
-    <row r="33" spans="1:8">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" s="94"/>
       <c r="B33" s="95"/>
       <c r="C33" s="95"/>
@@ -3586,7 +3597,7 @@
       <c r="F33" s="95"/>
       <c r="G33" s="96"/>
     </row>
-    <row r="34" spans="1:8">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" s="94"/>
       <c r="B34" s="95"/>
       <c r="C34" s="95"/>
@@ -3595,7 +3606,7 @@
       <c r="F34" s="95"/>
       <c r="G34" s="96"/>
     </row>
-    <row r="35" spans="1:8">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" s="94"/>
       <c r="B35" s="95"/>
       <c r="C35" s="95"/>
@@ -3604,7 +3615,7 @@
       <c r="F35" s="95"/>
       <c r="G35" s="96"/>
     </row>
-    <row r="36" spans="1:8">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" s="94"/>
       <c r="B36" s="95"/>
       <c r="C36" s="95"/>
@@ -3613,7 +3624,7 @@
       <c r="F36" s="95"/>
       <c r="G36" s="96"/>
     </row>
-    <row r="37" spans="1:8">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" s="94"/>
       <c r="B37" s="95"/>
       <c r="C37" s="95"/>
@@ -3622,7 +3633,7 @@
       <c r="F37" s="95"/>
       <c r="G37" s="96"/>
     </row>
-    <row r="38" spans="1:8">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" s="94"/>
       <c r="B38" s="95"/>
       <c r="C38" s="95"/>
@@ -3631,7 +3642,7 @@
       <c r="F38" s="95"/>
       <c r="G38" s="96"/>
     </row>
-    <row r="39" spans="1:8">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" s="94"/>
       <c r="B39" s="95"/>
       <c r="C39" s="95"/>
@@ -3641,7 +3652,7 @@
       <c r="G39" s="96"/>
       <c r="H39" s="67"/>
     </row>
-    <row r="40" spans="1:8">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="94"/>
       <c r="B40" s="95"/>
       <c r="C40" s="95"/>
@@ -3650,7 +3661,7 @@
       <c r="F40" s="95"/>
       <c r="G40" s="96"/>
     </row>
-    <row r="41" spans="1:8">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" s="94"/>
       <c r="B41" s="95"/>
       <c r="C41" s="95"/>
@@ -3659,7 +3670,7 @@
       <c r="F41" s="95"/>
       <c r="G41" s="96"/>
     </row>
-    <row r="42" spans="1:8">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" s="94"/>
       <c r="B42" s="95"/>
       <c r="C42" s="95"/>
@@ -3668,7 +3679,7 @@
       <c r="F42" s="95"/>
       <c r="G42" s="96"/>
     </row>
-    <row r="43" spans="1:8">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43" s="94"/>
       <c r="B43" s="95"/>
       <c r="C43" s="95"/>
@@ -3677,7 +3688,7 @@
       <c r="F43" s="95"/>
       <c r="G43" s="96"/>
     </row>
-    <row r="44" spans="1:8">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" s="94"/>
       <c r="B44" s="95"/>
       <c r="C44" s="95"/>
@@ -3686,7 +3697,7 @@
       <c r="F44" s="95"/>
       <c r="G44" s="96"/>
     </row>
-    <row r="45" spans="1:8" ht="13.5" thickBot="1">
+    <row r="45" spans="1:8" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A45" s="97"/>
       <c r="B45" s="98"/>
       <c r="C45" s="98"/>
@@ -3695,8 +3706,8 @@
       <c r="F45" s="98"/>
       <c r="G45" s="99"/>
     </row>
-    <row r="46" spans="1:8" ht="13.5" thickBot="1"/>
-    <row r="47" spans="1:8" ht="21" thickBot="1">
+    <row r="46" spans="1:8" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="1:8" ht="21" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="88" t="s">
         <v>30</v>
       </c>
@@ -3707,7 +3718,7 @@
       <c r="F47" s="89"/>
       <c r="G47" s="90"/>
     </row>
-    <row r="48" spans="1:8">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A48" s="91"/>
       <c r="B48" s="92"/>
       <c r="C48" s="92"/>
@@ -3716,7 +3727,7 @@
       <c r="F48" s="92"/>
       <c r="G48" s="93"/>
     </row>
-    <row r="49" spans="1:7">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" s="94"/>
       <c r="B49" s="95"/>
       <c r="C49" s="95"/>
@@ -3725,7 +3736,7 @@
       <c r="F49" s="95"/>
       <c r="G49" s="96"/>
     </row>
-    <row r="50" spans="1:7">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" s="94"/>
       <c r="B50" s="95"/>
       <c r="C50" s="95"/>
@@ -3734,7 +3745,7 @@
       <c r="F50" s="95"/>
       <c r="G50" s="96"/>
     </row>
-    <row r="51" spans="1:7">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" s="94"/>
       <c r="B51" s="95"/>
       <c r="C51" s="95"/>
@@ -3743,7 +3754,7 @@
       <c r="F51" s="95"/>
       <c r="G51" s="96"/>
     </row>
-    <row r="52" spans="1:7">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" s="94"/>
       <c r="B52" s="95"/>
       <c r="C52" s="95"/>
@@ -3752,7 +3763,7 @@
       <c r="F52" s="95"/>
       <c r="G52" s="96"/>
     </row>
-    <row r="53" spans="1:7">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" s="94"/>
       <c r="B53" s="95"/>
       <c r="C53" s="95"/>
@@ -3761,7 +3772,7 @@
       <c r="F53" s="95"/>
       <c r="G53" s="96"/>
     </row>
-    <row r="54" spans="1:7">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" s="94"/>
       <c r="B54" s="95"/>
       <c r="C54" s="95"/>
@@ -3770,7 +3781,7 @@
       <c r="F54" s="95"/>
       <c r="G54" s="96"/>
     </row>
-    <row r="55" spans="1:7">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" s="94"/>
       <c r="B55" s="95"/>
       <c r="C55" s="95"/>
@@ -3779,7 +3790,7 @@
       <c r="F55" s="95"/>
       <c r="G55" s="96"/>
     </row>
-    <row r="56" spans="1:7">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" s="94"/>
       <c r="B56" s="95"/>
       <c r="C56" s="95"/>
@@ -3788,7 +3799,7 @@
       <c r="F56" s="95"/>
       <c r="G56" s="96"/>
     </row>
-    <row r="57" spans="1:7">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57" s="94"/>
       <c r="B57" s="95"/>
       <c r="C57" s="95"/>
@@ -3797,7 +3808,7 @@
       <c r="F57" s="95"/>
       <c r="G57" s="96"/>
     </row>
-    <row r="58" spans="1:7">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A58" s="94"/>
       <c r="B58" s="95"/>
       <c r="C58" s="95"/>
@@ -3806,7 +3817,7 @@
       <c r="F58" s="95"/>
       <c r="G58" s="96"/>
     </row>
-    <row r="59" spans="1:7">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A59" s="94"/>
       <c r="B59" s="95"/>
       <c r="C59" s="95"/>
@@ -3815,7 +3826,7 @@
       <c r="F59" s="95"/>
       <c r="G59" s="96"/>
     </row>
-    <row r="60" spans="1:7">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A60" s="94"/>
       <c r="B60" s="95"/>
       <c r="C60" s="95"/>
@@ -3824,7 +3835,7 @@
       <c r="F60" s="95"/>
       <c r="G60" s="96"/>
     </row>
-    <row r="61" spans="1:7">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A61" s="94"/>
       <c r="B61" s="95"/>
       <c r="C61" s="95"/>
@@ -3833,7 +3844,7 @@
       <c r="F61" s="95"/>
       <c r="G61" s="96"/>
     </row>
-    <row r="62" spans="1:7">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A62" s="94"/>
       <c r="B62" s="95"/>
       <c r="C62" s="95"/>
@@ -3842,7 +3853,7 @@
       <c r="F62" s="95"/>
       <c r="G62" s="96"/>
     </row>
-    <row r="63" spans="1:7">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A63" s="94"/>
       <c r="B63" s="95"/>
       <c r="C63" s="95"/>
@@ -3851,7 +3862,7 @@
       <c r="F63" s="95"/>
       <c r="G63" s="96"/>
     </row>
-    <row r="64" spans="1:7">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A64" s="94"/>
       <c r="B64" s="95"/>
       <c r="C64" s="95"/>
@@ -3860,7 +3871,7 @@
       <c r="F64" s="95"/>
       <c r="G64" s="96"/>
     </row>
-    <row r="65" spans="1:7">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A65" s="94"/>
       <c r="B65" s="95"/>
       <c r="C65" s="95"/>
@@ -3869,7 +3880,7 @@
       <c r="F65" s="95"/>
       <c r="G65" s="96"/>
     </row>
-    <row r="66" spans="1:7">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A66" s="94"/>
       <c r="B66" s="95"/>
       <c r="C66" s="95"/>
@@ -3878,7 +3889,7 @@
       <c r="F66" s="95"/>
       <c r="G66" s="96"/>
     </row>
-    <row r="67" spans="1:7">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A67" s="94"/>
       <c r="B67" s="95"/>
       <c r="C67" s="95"/>
@@ -3887,7 +3898,7 @@
       <c r="F67" s="95"/>
       <c r="G67" s="96"/>
     </row>
-    <row r="68" spans="1:7">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A68" s="94"/>
       <c r="B68" s="95"/>
       <c r="C68" s="95"/>
@@ -3896,7 +3907,7 @@
       <c r="F68" s="95"/>
       <c r="G68" s="96"/>
     </row>
-    <row r="69" spans="1:7">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A69" s="94"/>
       <c r="B69" s="95"/>
       <c r="C69" s="95"/>
@@ -3905,7 +3916,7 @@
       <c r="F69" s="95"/>
       <c r="G69" s="96"/>
     </row>
-    <row r="70" spans="1:7">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A70" s="94"/>
       <c r="B70" s="95"/>
       <c r="C70" s="95"/>
@@ -3914,7 +3925,7 @@
       <c r="F70" s="95"/>
       <c r="G70" s="96"/>
     </row>
-    <row r="71" spans="1:7">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A71" s="94"/>
       <c r="B71" s="95"/>
       <c r="C71" s="95"/>
@@ -3923,7 +3934,7 @@
       <c r="F71" s="95"/>
       <c r="G71" s="96"/>
     </row>
-    <row r="72" spans="1:7">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A72" s="94"/>
       <c r="B72" s="95"/>
       <c r="C72" s="95"/>
@@ -3932,7 +3943,7 @@
       <c r="F72" s="95"/>
       <c r="G72" s="96"/>
     </row>
-    <row r="73" spans="1:7">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A73" s="94"/>
       <c r="B73" s="95"/>
       <c r="C73" s="95"/>
@@ -3941,7 +3952,7 @@
       <c r="F73" s="95"/>
       <c r="G73" s="96"/>
     </row>
-    <row r="74" spans="1:7">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A74" s="94"/>
       <c r="B74" s="95"/>
       <c r="C74" s="95"/>
@@ -3950,7 +3961,7 @@
       <c r="F74" s="95"/>
       <c r="G74" s="96"/>
     </row>
-    <row r="75" spans="1:7">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A75" s="94"/>
       <c r="B75" s="95"/>
       <c r="C75" s="95"/>
@@ -3959,7 +3970,7 @@
       <c r="F75" s="95"/>
       <c r="G75" s="96"/>
     </row>
-    <row r="76" spans="1:7">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A76" s="94"/>
       <c r="B76" s="95"/>
       <c r="C76" s="95"/>
@@ -3968,7 +3979,7 @@
       <c r="F76" s="95"/>
       <c r="G76" s="96"/>
     </row>
-    <row r="77" spans="1:7">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A77" s="94"/>
       <c r="B77" s="95"/>
       <c r="C77" s="95"/>
@@ -3977,7 +3988,7 @@
       <c r="F77" s="95"/>
       <c r="G77" s="96"/>
     </row>
-    <row r="78" spans="1:7">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A78" s="94"/>
       <c r="B78" s="95"/>
       <c r="C78" s="95"/>
@@ -3986,7 +3997,7 @@
       <c r="F78" s="95"/>
       <c r="G78" s="96"/>
     </row>
-    <row r="79" spans="1:7">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A79" s="94"/>
       <c r="B79" s="95"/>
       <c r="C79" s="95"/>
@@ -3995,7 +4006,7 @@
       <c r="F79" s="95"/>
       <c r="G79" s="96"/>
     </row>
-    <row r="80" spans="1:7">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A80" s="94"/>
       <c r="B80" s="95"/>
       <c r="C80" s="95"/>
@@ -4004,7 +4015,7 @@
       <c r="F80" s="95"/>
       <c r="G80" s="96"/>
     </row>
-    <row r="81" spans="1:7">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A81" s="94"/>
       <c r="B81" s="95"/>
       <c r="C81" s="95"/>
@@ -4013,7 +4024,7 @@
       <c r="F81" s="95"/>
       <c r="G81" s="96"/>
     </row>
-    <row r="82" spans="1:7">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A82" s="94"/>
       <c r="B82" s="95"/>
       <c r="C82" s="95"/>
@@ -4022,7 +4033,7 @@
       <c r="F82" s="95"/>
       <c r="G82" s="96"/>
     </row>
-    <row r="83" spans="1:7" ht="13.5" thickBot="1">
+    <row r="83" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A83" s="97"/>
       <c r="B83" s="98"/>
       <c r="C83" s="98"/>
@@ -4031,8 +4042,8 @@
       <c r="F83" s="98"/>
       <c r="G83" s="99"/>
     </row>
-    <row r="84" spans="1:7" ht="13.5" thickBot="1"/>
-    <row r="85" spans="1:7" ht="21" thickBot="1">
+    <row r="84" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="85" spans="1:7" ht="21" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A85" s="88" t="s">
         <v>31</v>
       </c>
@@ -4043,7 +4054,7 @@
       <c r="F85" s="89"/>
       <c r="G85" s="90"/>
     </row>
-    <row r="86" spans="1:7">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A86" s="91"/>
       <c r="B86" s="92"/>
       <c r="C86" s="92"/>
@@ -4052,7 +4063,7 @@
       <c r="F86" s="92"/>
       <c r="G86" s="93"/>
     </row>
-    <row r="87" spans="1:7">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A87" s="94"/>
       <c r="B87" s="95"/>
       <c r="C87" s="95"/>
@@ -4061,7 +4072,7 @@
       <c r="F87" s="95"/>
       <c r="G87" s="96"/>
     </row>
-    <row r="88" spans="1:7">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A88" s="94"/>
       <c r="B88" s="95"/>
       <c r="C88" s="95"/>
@@ -4070,7 +4081,7 @@
       <c r="F88" s="95"/>
       <c r="G88" s="96"/>
     </row>
-    <row r="89" spans="1:7">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A89" s="94"/>
       <c r="B89" s="95"/>
       <c r="C89" s="95"/>
@@ -4079,7 +4090,7 @@
       <c r="F89" s="95"/>
       <c r="G89" s="96"/>
     </row>
-    <row r="90" spans="1:7">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A90" s="94"/>
       <c r="B90" s="95"/>
       <c r="C90" s="95"/>
@@ -4088,7 +4099,7 @@
       <c r="F90" s="95"/>
       <c r="G90" s="96"/>
     </row>
-    <row r="91" spans="1:7">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A91" s="94"/>
       <c r="B91" s="95"/>
       <c r="C91" s="95"/>
@@ -4097,7 +4108,7 @@
       <c r="F91" s="95"/>
       <c r="G91" s="96"/>
     </row>
-    <row r="92" spans="1:7">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A92" s="94"/>
       <c r="B92" s="95"/>
       <c r="C92" s="95"/>
@@ -4106,7 +4117,7 @@
       <c r="F92" s="95"/>
       <c r="G92" s="96"/>
     </row>
-    <row r="93" spans="1:7">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A93" s="94"/>
       <c r="B93" s="95"/>
       <c r="C93" s="95"/>
@@ -4115,7 +4126,7 @@
       <c r="F93" s="95"/>
       <c r="G93" s="96"/>
     </row>
-    <row r="94" spans="1:7">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A94" s="94"/>
       <c r="B94" s="95"/>
       <c r="C94" s="95"/>
@@ -4124,7 +4135,7 @@
       <c r="F94" s="95"/>
       <c r="G94" s="96"/>
     </row>
-    <row r="95" spans="1:7">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A95" s="94"/>
       <c r="B95" s="95"/>
       <c r="C95" s="95"/>
@@ -4133,7 +4144,7 @@
       <c r="F95" s="95"/>
       <c r="G95" s="96"/>
     </row>
-    <row r="96" spans="1:7">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A96" s="94"/>
       <c r="B96" s="95"/>
       <c r="C96" s="95"/>
@@ -4142,7 +4153,7 @@
       <c r="F96" s="95"/>
       <c r="G96" s="96"/>
     </row>
-    <row r="97" spans="1:7">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A97" s="94"/>
       <c r="B97" s="95"/>
       <c r="C97" s="95"/>
@@ -4151,7 +4162,7 @@
       <c r="F97" s="95"/>
       <c r="G97" s="96"/>
     </row>
-    <row r="98" spans="1:7">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A98" s="94"/>
       <c r="B98" s="95"/>
       <c r="C98" s="95"/>
@@ -4160,7 +4171,7 @@
       <c r="F98" s="95"/>
       <c r="G98" s="96"/>
     </row>
-    <row r="99" spans="1:7">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A99" s="94"/>
       <c r="B99" s="95"/>
       <c r="C99" s="95"/>
@@ -4169,7 +4180,7 @@
       <c r="F99" s="95"/>
       <c r="G99" s="96"/>
     </row>
-    <row r="100" spans="1:7">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A100" s="94"/>
       <c r="B100" s="95"/>
       <c r="C100" s="95"/>
@@ -4178,7 +4189,7 @@
       <c r="F100" s="95"/>
       <c r="G100" s="96"/>
     </row>
-    <row r="101" spans="1:7">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A101" s="94"/>
       <c r="B101" s="95"/>
       <c r="C101" s="95"/>
@@ -4187,7 +4198,7 @@
       <c r="F101" s="95"/>
       <c r="G101" s="96"/>
     </row>
-    <row r="102" spans="1:7">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A102" s="94"/>
       <c r="B102" s="95"/>
       <c r="C102" s="95"/>
@@ -4196,7 +4207,7 @@
       <c r="F102" s="95"/>
       <c r="G102" s="96"/>
     </row>
-    <row r="103" spans="1:7">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A103" s="94"/>
       <c r="B103" s="95"/>
       <c r="C103" s="95"/>
@@ -4205,7 +4216,7 @@
       <c r="F103" s="95"/>
       <c r="G103" s="96"/>
     </row>
-    <row r="104" spans="1:7">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A104" s="94"/>
       <c r="B104" s="95"/>
       <c r="C104" s="95"/>
@@ -4214,7 +4225,7 @@
       <c r="F104" s="95"/>
       <c r="G104" s="96"/>
     </row>
-    <row r="105" spans="1:7">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A105" s="94"/>
       <c r="B105" s="95"/>
       <c r="C105" s="95"/>
@@ -4223,7 +4234,7 @@
       <c r="F105" s="95"/>
       <c r="G105" s="96"/>
     </row>
-    <row r="106" spans="1:7">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A106" s="94"/>
       <c r="B106" s="95"/>
       <c r="C106" s="95"/>
@@ -4232,7 +4243,7 @@
       <c r="F106" s="95"/>
       <c r="G106" s="96"/>
     </row>
-    <row r="107" spans="1:7">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A107" s="94"/>
       <c r="B107" s="95"/>
       <c r="C107" s="95"/>
@@ -4241,7 +4252,7 @@
       <c r="F107" s="95"/>
       <c r="G107" s="96"/>
     </row>
-    <row r="108" spans="1:7">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A108" s="94"/>
       <c r="B108" s="95"/>
       <c r="C108" s="95"/>
@@ -4250,7 +4261,7 @@
       <c r="F108" s="95"/>
       <c r="G108" s="96"/>
     </row>
-    <row r="109" spans="1:7">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A109" s="94"/>
       <c r="B109" s="95"/>
       <c r="C109" s="95"/>
@@ -4259,7 +4270,7 @@
       <c r="F109" s="95"/>
       <c r="G109" s="96"/>
     </row>
-    <row r="110" spans="1:7">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A110" s="94"/>
       <c r="B110" s="95"/>
       <c r="C110" s="95"/>
@@ -4268,7 +4279,7 @@
       <c r="F110" s="95"/>
       <c r="G110" s="96"/>
     </row>
-    <row r="111" spans="1:7">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A111" s="94"/>
       <c r="B111" s="95"/>
       <c r="C111" s="95"/>
@@ -4277,7 +4288,7 @@
       <c r="F111" s="95"/>
       <c r="G111" s="96"/>
     </row>
-    <row r="112" spans="1:7">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A112" s="94"/>
       <c r="B112" s="95"/>
       <c r="C112" s="95"/>
@@ -4286,7 +4297,7 @@
       <c r="F112" s="95"/>
       <c r="G112" s="96"/>
     </row>
-    <row r="113" spans="1:7">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A113" s="94"/>
       <c r="B113" s="95"/>
       <c r="C113" s="95"/>
@@ -4295,7 +4306,7 @@
       <c r="F113" s="95"/>
       <c r="G113" s="96"/>
     </row>
-    <row r="114" spans="1:7">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A114" s="94"/>
       <c r="B114" s="95"/>
       <c r="C114" s="95"/>
@@ -4304,7 +4315,7 @@
       <c r="F114" s="95"/>
       <c r="G114" s="96"/>
     </row>
-    <row r="115" spans="1:7">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A115" s="94"/>
       <c r="B115" s="95"/>
       <c r="C115" s="95"/>
@@ -4313,7 +4324,7 @@
       <c r="F115" s="95"/>
       <c r="G115" s="96"/>
     </row>
-    <row r="116" spans="1:7">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A116" s="94"/>
       <c r="B116" s="95"/>
       <c r="C116" s="95"/>
@@ -4322,7 +4333,7 @@
       <c r="F116" s="95"/>
       <c r="G116" s="96"/>
     </row>
-    <row r="117" spans="1:7">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A117" s="94"/>
       <c r="B117" s="95"/>
       <c r="C117" s="95"/>
@@ -4331,7 +4342,7 @@
       <c r="F117" s="95"/>
       <c r="G117" s="96"/>
     </row>
-    <row r="118" spans="1:7">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A118" s="94"/>
       <c r="B118" s="95"/>
       <c r="C118" s="95"/>
@@ -4340,7 +4351,7 @@
       <c r="F118" s="95"/>
       <c r="G118" s="96"/>
     </row>
-    <row r="119" spans="1:7">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A119" s="94"/>
       <c r="B119" s="95"/>
       <c r="C119" s="95"/>
@@ -4349,7 +4360,7 @@
       <c r="F119" s="95"/>
       <c r="G119" s="96"/>
     </row>
-    <row r="120" spans="1:7">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A120" s="94"/>
       <c r="B120" s="95"/>
       <c r="C120" s="95"/>
@@ -4358,7 +4369,7 @@
       <c r="F120" s="95"/>
       <c r="G120" s="96"/>
     </row>
-    <row r="121" spans="1:7" ht="13.5" thickBot="1">
+    <row r="121" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A121" s="97"/>
       <c r="B121" s="98"/>
       <c r="C121" s="98"/>
@@ -4368,7 +4379,7 @@
       <c r="G121" s="99"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="eL9sw/aSPfocmfa5jx8e2xa9v0XIBIliIwFWTooRXK1YTH3QJYozL/OBY7cao5bu6dDA+85tJ3ic0293xTQX5w==" saltValue="clEHaHehhbGKCh5Lrevn2Q==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <mergeCells count="7">
     <mergeCell ref="A2:G6"/>
     <mergeCell ref="A85:G85"/>
@@ -4379,7 +4390,8 @@
     <mergeCell ref="A48:G83"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -4389,49 +4401,49 @@
     <tabColor theme="9"/>
   </sheetPr>
   <dimension ref="A1:K155"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.85546875" customWidth="1"/>
     <col min="2" max="2" width="38.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="35.25">
+    <row r="1" spans="1:11" ht="35.25" x14ac:dyDescent="0.2">
       <c r="A1" s="102" t="s">
         <v>34</v>
       </c>
       <c r="B1" s="102"/>
       <c r="C1" s="102"/>
       <c r="D1" s="102"/>
-      <c r="E1" s="102"/>
-      <c r="F1" s="102"/>
-      <c r="G1" s="102"/>
-    </row>
-    <row r="2" spans="1:11" ht="23.25">
+      <c r="E1" s="106"/>
+      <c r="F1" s="106"/>
+      <c r="G1" s="106"/>
+    </row>
+    <row r="2" spans="1:11" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A2" s="103" t="s">
         <v>35</v>
       </c>
       <c r="B2" s="103"/>
       <c r="C2" s="103"/>
       <c r="D2" s="103"/>
-      <c r="E2" s="103"/>
-      <c r="F2" s="103"/>
-      <c r="G2" s="103"/>
-    </row>
-    <row r="3" spans="1:11" ht="23.25">
+      <c r="E2" s="107"/>
+      <c r="F2" s="107"/>
+      <c r="G2" s="107"/>
+    </row>
+    <row r="3" spans="1:11" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A3" s="103" t="s">
         <v>36</v>
       </c>
       <c r="B3" s="103"/>
       <c r="C3" s="103"/>
       <c r="D3" s="103"/>
-      <c r="E3" s="103"/>
-      <c r="F3" s="103"/>
-      <c r="G3" s="103"/>
-    </row>
-    <row r="4" spans="1:11" ht="13.5" thickBot="1">
+      <c r="E3" s="107"/>
+      <c r="F3" s="107"/>
+      <c r="G3" s="107"/>
+    </row>
+    <row r="4" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="13"/>
     </row>
-    <row r="5" spans="1:11" ht="15.75" thickBot="1">
+    <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>37</v>
       </c>
@@ -4439,7 +4451,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16.5" thickTop="1" thickBot="1">
+    <row r="6" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
         <v>39</v>
       </c>
@@ -4447,7 +4459,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15.75" thickBot="1">
+    <row r="7" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">
         <v>41</v>
       </c>
@@ -4455,23 +4467,23 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="18.75">
+    <row r="8" spans="1:11" ht="18.75" x14ac:dyDescent="0.2">
       <c r="A8" s="20" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="17.25">
+    <row r="9" spans="1:11" ht="17.25" x14ac:dyDescent="0.2">
       <c r="A9" s="21" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="73.5" customHeight="1">
-      <c r="A10" s="104" t="s">
+    <row r="10" spans="1:11" ht="83.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="105" t="s">
         <v>44</v>
       </c>
-      <c r="B10" s="104"/>
-      <c r="C10" s="104"/>
-      <c r="D10" s="104"/>
+      <c r="B10" s="105"/>
+      <c r="C10" s="105"/>
+      <c r="D10" s="105"/>
       <c r="E10" s="104"/>
       <c r="F10" s="104"/>
       <c r="G10" s="104"/>
@@ -4480,12 +4492,12 @@
       <c r="J10" s="104"/>
       <c r="K10" s="104"/>
     </row>
-    <row r="11" spans="1:11" ht="17.25">
+    <row r="11" spans="1:11" ht="17.25" x14ac:dyDescent="0.2">
       <c r="A11" s="21" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="15">
+    <row r="12" spans="1:11" ht="15" x14ac:dyDescent="0.2">
       <c r="A12" s="46" t="s">
         <v>46</v>
       </c>
@@ -4493,71 +4505,71 @@
       <c r="C12" s="47"/>
       <c r="D12" s="47"/>
     </row>
-    <row r="13" spans="1:11" s="1" customFormat="1" ht="15">
+    <row r="13" spans="1:11" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A13" s="46"/>
       <c r="B13" s="47"/>
       <c r="C13" s="47"/>
       <c r="D13" s="47"/>
     </row>
-    <row r="14" spans="1:11" ht="14.25">
+    <row r="14" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A14" s="23" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="14.25">
+    <row r="15" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A15" s="23" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="14.25">
+    <row r="16" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A16" s="23" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="14.25">
+    <row r="17" spans="1:2" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A17" s="23" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="14.25">
+    <row r="18" spans="1:2" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A18" s="23" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="14.25">
+    <row r="19" spans="1:2" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A19" s="23" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="14.25">
+    <row r="20" spans="1:2" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A20" s="23" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="14.25">
+    <row r="21" spans="1:2" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A21" s="23" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="14.25">
+    <row r="22" spans="1:2" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A22" s="23" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="23" spans="1:2" s="1" customFormat="1" ht="14.25">
+    <row r="23" spans="1:2" s="1" customFormat="1" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A23" s="23"/>
     </row>
-    <row r="24" spans="1:2" ht="18.75">
+    <row r="24" spans="1:2" ht="18.75" x14ac:dyDescent="0.2">
       <c r="A24" s="20" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="18" thickBot="1">
+    <row r="25" spans="1:2" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="21" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="15.75" thickBot="1">
+    <row r="26" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A26" s="24" t="s">
         <v>58</v>
       </c>
@@ -4565,7 +4577,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="52.5" customHeight="1" thickTop="1" thickBot="1">
+    <row r="27" spans="1:2" ht="52.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" s="25" t="s">
         <v>59</v>
       </c>
@@ -4573,123 +4585,126 @@
         <v>60</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="15">
+    <row r="29" spans="1:2" ht="15" x14ac:dyDescent="0.2">
       <c r="A29" s="27" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="30" spans="1:2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" s="28" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="31" spans="1:2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" s="28" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="32" spans="1:2" s="1" customFormat="1">
+    <row r="32" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A32" s="28"/>
     </row>
-    <row r="33" spans="1:1" ht="15">
+    <row r="33" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A33" s="27" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="34" spans="1:1">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" s="28" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="35" spans="1:1">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" s="28" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="36" spans="1:1" s="1" customFormat="1">
+    <row r="36" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="28"/>
     </row>
-    <row r="37" spans="1:1" ht="17.25">
+    <row r="37" spans="1:4" ht="17.25" x14ac:dyDescent="0.2">
       <c r="A37" s="21" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="38" spans="1:1" ht="14.25">
+    <row r="38" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A38" s="22" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="39" spans="1:1" s="1" customFormat="1" ht="14.25">
+    <row r="39" spans="1:4" s="1" customFormat="1" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A39" s="22"/>
     </row>
-    <row r="40" spans="1:1" ht="15">
+    <row r="40" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A40" s="27" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="41" spans="1:1">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" s="28" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="42" spans="1:1">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" s="28" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="43" spans="1:1">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" s="28" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="44" spans="1:1" s="1" customFormat="1">
+    <row r="44" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A44" s="28"/>
     </row>
-    <row r="45" spans="1:1" ht="17.25">
+    <row r="45" spans="1:4" ht="17.25" x14ac:dyDescent="0.2">
       <c r="A45" s="21" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="46" spans="1:1">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" s="29" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="47" spans="1:1">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" s="29" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="48" spans="1:1">
-      <c r="A48" s="29" t="s">
+    <row r="48" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="108" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="49" spans="1:2" s="1" customFormat="1">
+      <c r="B48" s="108"/>
+      <c r="C48" s="108"/>
+      <c r="D48" s="108"/>
+    </row>
+    <row r="49" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A49" s="29"/>
     </row>
-    <row r="50" spans="1:2" ht="18.75">
+    <row r="50" spans="1:2" ht="18.75" x14ac:dyDescent="0.2">
       <c r="A50" s="20" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="51" spans="1:2" s="1" customFormat="1" ht="18.75">
+    <row r="51" spans="1:2" s="1" customFormat="1" ht="18.75" x14ac:dyDescent="0.2">
       <c r="A51" s="20"/>
     </row>
-    <row r="52" spans="1:2" ht="17.25">
+    <row r="52" spans="1:2" ht="17.25" x14ac:dyDescent="0.2">
       <c r="A52" s="21" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="53" spans="1:2" s="1" customFormat="1" ht="17.25">
+    <row r="53" spans="1:2" s="1" customFormat="1" ht="17.25" x14ac:dyDescent="0.2">
       <c r="A53" s="21"/>
     </row>
-    <row r="54" spans="1:2" ht="15" thickBot="1">
+    <row r="54" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="22" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="55" spans="1:2" ht="15.75" thickBot="1">
+    <row r="55" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A55" s="24" t="s">
         <v>79</v>
       </c>
@@ -4697,7 +4712,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="1:2" ht="14.25" thickTop="1" thickBot="1">
+    <row r="56" spans="1:2" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A56" s="25" t="s">
         <v>80</v>
       </c>
@@ -4705,7 +4720,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="57" spans="1:2" ht="13.5" thickBot="1">
+    <row r="57" spans="1:2" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A57" s="30" t="s">
         <v>82</v>
       </c>
@@ -4713,7 +4728,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="58" spans="1:2" ht="13.5" thickBot="1">
+    <row r="58" spans="1:2" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A58" s="32" t="s">
         <v>84</v>
       </c>
@@ -4721,73 +4736,73 @@
         <v>85</v>
       </c>
     </row>
-    <row r="60" spans="1:2" ht="15">
+    <row r="60" spans="1:2" ht="15" x14ac:dyDescent="0.2">
       <c r="A60" s="34" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="61" spans="1:2">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A61" s="11" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="62" spans="1:2">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A62" s="29" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="63" spans="1:2">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A63" s="28" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="64" spans="1:2">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A64" s="28" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="65" spans="1:2">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A65" s="28" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="66" spans="1:2">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A66" s="28" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="67" spans="1:2" s="1" customFormat="1">
+    <row r="67" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A67" s="28"/>
     </row>
-    <row r="68" spans="1:2" ht="17.25">
+    <row r="68" spans="1:2" ht="17.25" x14ac:dyDescent="0.2">
       <c r="A68" s="21" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="69" spans="1:2">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A69" s="28" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="70" spans="1:2">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A70" s="28" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="71" spans="1:2" s="1" customFormat="1">
+    <row r="71" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A71" s="28"/>
     </row>
-    <row r="72" spans="1:2" ht="14.25">
+    <row r="72" spans="1:2" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A72" s="35" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="73" spans="1:2" ht="18" thickBot="1">
+    <row r="73" spans="1:2" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A73" s="21" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="74" spans="1:2" ht="15.75" thickBot="1">
+    <row r="74" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A74" s="24" t="s">
         <v>58</v>
       </c>
@@ -4795,7 +4810,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="75" spans="1:2" ht="14.25" thickTop="1" thickBot="1">
+    <row r="75" spans="1:2" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A75" s="25" t="s">
         <v>59</v>
       </c>
@@ -4803,7 +4818,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="76" spans="1:2" ht="13.5" thickBot="1">
+    <row r="76" spans="1:2" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A76" s="30" t="s">
         <v>100</v>
       </c>
@@ -4811,7 +4826,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="77" spans="1:2">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A77" s="100" t="s">
         <v>102</v>
       </c>
@@ -4819,163 +4834,163 @@
         <v>103</v>
       </c>
     </row>
-    <row r="78" spans="1:2" ht="13.5" thickBot="1">
+    <row r="78" spans="1:2" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A78" s="101"/>
       <c r="B78" s="37" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="80" spans="1:2" ht="15">
+    <row r="80" spans="1:2" ht="15" x14ac:dyDescent="0.2">
       <c r="A80" s="27" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="81" spans="1:1">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A81" s="28" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="82" spans="1:1">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A82" s="28" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="83" spans="1:1" s="1" customFormat="1">
+    <row r="83" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A83" s="28"/>
     </row>
-    <row r="84" spans="1:1" ht="17.25">
+    <row r="84" spans="1:1" ht="17.25" x14ac:dyDescent="0.2">
       <c r="A84" s="21" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="85" spans="1:1" ht="14.25">
+    <row r="85" spans="1:1" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A85" s="22" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="86" spans="1:1">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A86" s="28" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="87" spans="1:1">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A87" s="28" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="88" spans="1:1">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A88" s="28" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="89" spans="1:1" s="1" customFormat="1">
+    <row r="89" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A89" s="28"/>
     </row>
-    <row r="90" spans="1:1" ht="17.25">
+    <row r="90" spans="1:1" ht="17.25" x14ac:dyDescent="0.2">
       <c r="A90" s="21" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="91" spans="1:1">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A91" s="29" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="92" spans="1:1">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A92" s="29" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="93" spans="1:1" s="1" customFormat="1">
+    <row r="93" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A93" s="29"/>
     </row>
-    <row r="94" spans="1:1" ht="17.25">
+    <row r="94" spans="1:1" ht="17.25" x14ac:dyDescent="0.2">
       <c r="A94" s="21" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="95" spans="1:1" s="1" customFormat="1" ht="17.25">
+    <row r="95" spans="1:1" s="1" customFormat="1" ht="17.25" x14ac:dyDescent="0.2">
       <c r="A95" s="21"/>
     </row>
-    <row r="96" spans="1:1" ht="15">
+    <row r="96" spans="1:1" ht="15" x14ac:dyDescent="0.2">
       <c r="A96" s="34" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="97" spans="1:1">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A97" s="11" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="99" spans="1:1" ht="15">
+    <row r="99" spans="1:1" ht="15" x14ac:dyDescent="0.2">
       <c r="A99" s="27" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="100" spans="1:1">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A100" s="28" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="101" spans="1:1">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A101" s="28" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="102" spans="1:1" ht="15">
+    <row r="102" spans="1:1" ht="15" x14ac:dyDescent="0.2">
       <c r="A102" s="27" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="103" spans="1:1">
+    <row r="103" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A103" s="28" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="104" spans="1:1">
+    <row r="104" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A104" s="28" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="105" spans="1:1">
+    <row r="105" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A105" s="28" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="106" spans="1:1" ht="15">
+    <row r="106" spans="1:1" ht="15" x14ac:dyDescent="0.2">
       <c r="A106" s="27" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="107" spans="1:1">
+    <row r="107" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A107" s="28" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="108" spans="1:1">
+    <row r="108" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A108" s="28" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="109" spans="1:1">
+    <row r="109" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A109" s="28" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="110" spans="1:1" s="1" customFormat="1">
+    <row r="110" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A110" s="28"/>
     </row>
-    <row r="111" spans="1:1" ht="18.75">
+    <row r="111" spans="1:1" ht="18.75" x14ac:dyDescent="0.2">
       <c r="A111" s="20" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="112" spans="1:1" ht="18" thickBot="1">
+    <row r="112" spans="1:1" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A112" s="21" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="113" spans="1:2" ht="15.75" thickBot="1">
+    <row r="113" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A113" s="24" t="s">
         <v>131</v>
       </c>
@@ -4983,7 +4998,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="114" spans="1:2" ht="27" thickTop="1" thickBot="1">
+    <row r="114" spans="1:2" ht="27" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A114" s="25" t="s">
         <v>133</v>
       </c>
@@ -4991,7 +5006,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="115" spans="1:2" ht="13.5" thickBot="1">
+    <row r="115" spans="1:2" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A115" s="30" t="s">
         <v>135</v>
       </c>
@@ -4999,7 +5014,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="116" spans="1:2" ht="13.5" thickBot="1">
+    <row r="116" spans="1:2" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A116" s="32" t="s">
         <v>137</v>
       </c>
@@ -5007,33 +5022,33 @@
         <v>138</v>
       </c>
     </row>
-    <row r="118" spans="1:2">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A118" s="29" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="119" spans="1:2" s="1" customFormat="1">
+    <row r="119" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A119" s="29"/>
     </row>
-    <row r="120" spans="1:2" ht="18.75">
+    <row r="120" spans="1:2" ht="18.75" x14ac:dyDescent="0.2">
       <c r="A120" s="20" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="121" spans="1:2" ht="17.25">
+    <row r="121" spans="1:2" ht="17.25" x14ac:dyDescent="0.2">
       <c r="A121" s="21" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="122" spans="1:2">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A122" s="29" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="123" spans="1:2" ht="13.5" thickBot="1">
+    <row r="123" spans="1:2" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A123" s="13"/>
     </row>
-    <row r="124" spans="1:2" ht="15.75" thickBot="1">
+    <row r="124" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A124" s="38" t="s">
         <v>143</v>
       </c>
@@ -5041,7 +5056,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="125" spans="1:2" ht="14.25" thickTop="1" thickBot="1">
+    <row r="125" spans="1:2" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A125" s="39" t="s">
         <v>145</v>
       </c>
@@ -5049,7 +5064,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="126" spans="1:2" ht="13.5" thickBot="1">
+    <row r="126" spans="1:2" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A126" s="41" t="s">
         <v>146</v>
       </c>
@@ -5057,7 +5072,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="127" spans="1:2" ht="13.5" thickBot="1">
+    <row r="127" spans="1:2" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A127" s="43" t="s">
         <v>147</v>
       </c>
@@ -5065,148 +5080,150 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="129" spans="1:1">
+    <row r="129" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A129" s="29" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="130" spans="1:1" ht="15">
+    <row r="130" spans="1:1" ht="15" x14ac:dyDescent="0.2">
       <c r="A130" s="27" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="131" spans="1:1">
+    <row r="131" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A131" s="28" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="132" spans="1:1">
+    <row r="132" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A132" s="28" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="133" spans="1:1" s="1" customFormat="1">
+    <row r="133" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A133" s="28"/>
     </row>
-    <row r="134" spans="1:1" ht="18.75">
+    <row r="134" spans="1:1" ht="18.75" x14ac:dyDescent="0.2">
       <c r="A134" s="20" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="135" spans="1:1" ht="17.25">
+    <row r="135" spans="1:1" ht="17.25" x14ac:dyDescent="0.2">
       <c r="A135" s="21" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="136" spans="1:1">
+    <row r="136" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A136" s="28" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="137" spans="1:1">
+    <row r="137" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A137" s="28" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="138" spans="1:1" ht="17.25">
+    <row r="138" spans="1:1" ht="17.25" x14ac:dyDescent="0.2">
       <c r="A138" s="21" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="139" spans="1:1">
+    <row r="139" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A139" s="28" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="140" spans="1:1">
+    <row r="140" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A140" s="28" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="141" spans="1:1" ht="17.25">
+    <row r="141" spans="1:1" ht="17.25" x14ac:dyDescent="0.2">
       <c r="A141" s="21" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="142" spans="1:1">
+    <row r="142" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A142" s="28" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="143" spans="1:1">
+    <row r="143" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A143" s="45" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="144" spans="1:1">
+    <row r="144" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A144" s="28" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="145" spans="1:1">
+    <row r="145" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A145" s="28" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="146" spans="1:1">
+    <row r="146" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A146" s="28" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="147" spans="1:1">
+    <row r="147" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A147" s="28" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="148" spans="1:1">
+    <row r="148" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A148" s="45" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="149" spans="1:1">
+    <row r="149" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A149" s="28" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="150" spans="1:1">
+    <row r="150" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A150" s="11" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="151" spans="1:1">
+    <row r="151" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A151" s="28" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="152" spans="1:1">
+    <row r="152" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A152" s="28" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="153" spans="1:1">
+    <row r="153" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A153" s="28" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="154" spans="1:1">
+    <row r="154" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A154" s="28" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="155" spans="1:1">
+    <row r="155" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A155" s="28" t="s">
         <v>173</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="mv1pM/0r6OmolenHID3ibUIOOcgfqHYDf03nb0u063hVyxidZK5fNmzFHgmecISe0XbqZMPjIVKc6MzgE6q0sA==" saltValue="WsWkIuJ4T5wWb+SDxozp/Q==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
-  <mergeCells count="5">
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
+  <mergeCells count="6">
     <mergeCell ref="A77:A78"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A10:K10"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A48:D48"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>